<commit_message>
cleanup lint downto 8
</commit_message>
<xml_diff>
--- a/grisha/exported_data.xlsx
+++ b/grisha/exported_data.xlsx
@@ -94,10 +94,18 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,6 +473,16 @@
   </sheetPr>
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.2" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="9.6" customWidth="1" min="3" max="3"/>
+    <col width="13.2" customWidth="1" min="4" max="4"/>
+    <col width="8.4" customWidth="1" min="5" max="5"/>
+    <col width="14.4" customWidth="1" min="6" max="6"/>
+    <col width="20.4" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -549,6 +567,10 @@
   </sheetPr>
   <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16.8" customWidth="1" min="1" max="1"/>
+    <col width="20.4" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">

</xml_diff>